<commit_message>
update with better schedule code to reveal gradually
</commit_message>
<xml_diff>
--- a/ids540_specific/class_schedule_540_xlsx.xlsx
+++ b/ids540_specific/class_schedule_540_xlsx.xlsx
@@ -511,7 +511,7 @@
     <row r="2" ht="139" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tues, Aug 25</t>
+          <t>Mon, Aug 24</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -536,7 +536,7 @@
     <row r="3" ht="204" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Thurs, Aug 27</t>
+          <t>Wed, Aug 26</t>
         </is>
       </c>
       <c r="B3" s="11" t="inlineStr">
@@ -561,7 +561,7 @@
     <row r="4" ht="85" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Tues, Sep 1</t>
+          <t>Mon, Aug 31</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
@@ -589,7 +589,7 @@
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Thurs, Sep 3</t>
+          <t>Wed, Sep 2</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
@@ -612,7 +612,7 @@
     <row r="6" ht="51" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Tues, Sep 8</t>
+          <t>Mon, Sep 7</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
@@ -635,7 +635,7 @@
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Thurs, Sep 10</t>
+          <t>Wed, Sep 9</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
@@ -657,7 +657,7 @@
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Tues, Sep 15</t>
+          <t>Mon, Sep 14</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
@@ -679,7 +679,7 @@
     <row r="9" ht="118" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Thurs, Sep 17</t>
+          <t>Wed, Sep 16</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
@@ -696,7 +696,7 @@
     <row r="10" ht="51" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Tues, Sep 22</t>
+          <t>Mon, Sep 21</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
@@ -720,7 +720,7 @@
     <row r="11" ht="17" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Thurs, Sep 24</t>
+          <t>Wed, Sep 23</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Tues, Sep 29</t>
+          <t>Mon, Sep 28</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
@@ -759,7 +759,7 @@
     <row r="13" ht="136" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>Thurs, Oct 1</t>
+          <t>Wed, Sep 30</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -791,7 +791,7 @@
     <row r="14" ht="57" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>Tues, Oct 6</t>
+          <t>Mon, Oct 5</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -815,7 +815,7 @@
     <row r="15" ht="170" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Thurs, Oct 8</t>
+          <t>Wed, Oct 7</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
@@ -844,7 +844,7 @@
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Tues, Oct 13 (Break)</t>
+          <t>Mon, Oct 12 (Break)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -856,7 +856,7 @@
     <row r="17" ht="68" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Thurs, Oct 15 (Break)</t>
+          <t>Wed, Oct 14 (Break)</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
@@ -879,7 +879,7 @@
     <row r="18" ht="57" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Tues, Oct 20</t>
+          <t>Mon, Oct 19</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -903,7 +903,7 @@
     <row r="19" ht="85" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>Thurs, Oct 22</t>
+          <t>Wed, Oct 21</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
@@ -928,7 +928,7 @@
     <row r="20" ht="85" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Tues, Oct 27</t>
+          <t>Mon, Oct 26</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -954,7 +954,7 @@
     <row r="21" ht="106" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Thurs, Oct 29</t>
+          <t>Wed, Oct 28</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -978,7 +978,7 @@
     <row r="22" ht="140" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Tues, Nov 3</t>
+          <t>Mon, Nov 2</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -1003,7 +1003,7 @@
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Thurs, Nov 5</t>
+          <t>Wed, Nov 4</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
@@ -1020,7 +1020,7 @@
     <row r="24" ht="134" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Tues, Nov 10</t>
+          <t>Mon, Nov 9</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1047,7 +1047,7 @@
     <row r="25" ht="103" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>Thurs, Nov 12</t>
+          <t>Wed, Nov 11</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
@@ -1074,7 +1074,7 @@
     <row r="26" ht="105" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Tues, Nov 17</t>
+          <t>Mon, Nov 16</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1102,7 +1102,7 @@
     <row r="27" ht="43" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>Thurs, Nov 19</t>
+          <t>Wed, Nov 18</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">

</xml_diff>

<commit_message>
update for labor day and delayed triangle
</commit_message>
<xml_diff>
--- a/ids540_specific/class_schedule_540_xlsx.xlsx
+++ b/ids540_specific/class_schedule_540_xlsx.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vesper/Documents/GitHub/practicaldatascience_book/ids540_specific/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nce8/github/practicaldatascience_book/ids540_specific/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9A1787B-6FEF-F34C-8873-FB9B294DBA11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F60D1E2E-A11F-3F4F-9BAC-84D80F9295D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="34560" windowHeight="19460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="class_schedule_590" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="103">
   <si>
     <t>Date, Rm</t>
   </si>
@@ -360,15 +360,6 @@
     <t>Wed, Nov 18</t>
   </si>
   <si>
-    <t>- Statistics with statsmodels</t>
-  </si>
-  <si>
-    <t>- Read all readings under the Statistical Modelling heading, starting with `Inference and Prediction &lt;../notebooks/class_5/week_3/20_inference_v_prediction.html&gt;`_ through `Beyond the Basic Model &lt;../notebooks/class_5/week_3/40_linear_regression_extensions&gt;`_</t>
-  </si>
-  <si>
-    <t>- `Link &lt;../exercises/exercise_statsmodels.html&gt;`_</t>
-  </si>
-  <si>
     <t>Wed Dec 9</t>
   </si>
   <si>
@@ -395,6 +386,18 @@
     <t>- Using VS Code
 - `Max &lt;../exercises/exercises/20_max.html&gt;`_
 - `Triangle &lt;../exercises/exercises/30_triangle.html&gt;`_</t>
+  </si>
+  <si>
+    <t>LABOR DAY</t>
+  </si>
+  <si>
+    <t>Mon, Nov 23rd</t>
+  </si>
+  <si>
+    <t>Wed, Nov 25th</t>
+  </si>
+  <si>
+    <t>More time on Max and Triangle</t>
   </si>
 </sst>
 </file>
@@ -503,9 +506,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -543,7 +546,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -649,7 +652,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -791,7 +794,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -799,7 +802,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33.1640625" customWidth="1"/>
@@ -830,7 +833,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D2" s="7"/>
     </row>
@@ -853,10 +856,10 @@
         <v>10</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -870,35 +873,26 @@
         <v>12</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>16</v>
+      <c r="B6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C6" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>20</v>
+      <c r="B7" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -906,13 +900,13 @@
         <v>25</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="118" customHeight="1" x14ac:dyDescent="0.2">
@@ -920,13 +914,13 @@
         <v>29</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>28</v>
+        <v>19</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -934,10 +928,13 @@
         <v>32</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" t="s">
-        <v>31</v>
+        <v>22</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -945,13 +942,13 @@
         <v>36</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>35</v>
+        <v>27</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -959,10 +956,10 @@
         <v>38</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>37</v>
+        <v>30</v>
+      </c>
+      <c r="D12" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="136" customHeight="1" x14ac:dyDescent="0.2">
@@ -973,38 +970,35 @@
         <v>33</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="57" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>44</v>
+      <c r="B14" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="170" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>48</v>
+      <c r="B15" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
@@ -1017,16 +1011,16 @@
     </row>
     <row r="17" spans="1:4" ht="68" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>51</v>
+        <v>97</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="57" customHeight="1" x14ac:dyDescent="0.2">
@@ -1034,13 +1028,13 @@
         <v>57</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>56</v>
+        <v>46</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="85" customHeight="1" x14ac:dyDescent="0.2">
@@ -1048,13 +1042,13 @@
         <v>61</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>60</v>
+        <v>46</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="85" customHeight="1" x14ac:dyDescent="0.2">
@@ -1062,13 +1056,13 @@
         <v>65</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>64</v>
+        <v>54</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="106" customHeight="1" x14ac:dyDescent="0.2">
@@ -1076,66 +1070,69 @@
         <v>69</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>68</v>
+        <v>59</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="140" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="B22" s="3" t="s">
-        <v>70</v>
+      <c r="B22" s="6" t="s">
+        <v>62</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="60" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="85" x14ac:dyDescent="0.2">
       <c r="A23" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="B23" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>75</v>
+      <c r="B23" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>67</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="134" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="B24" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>78</v>
+      <c r="B24" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="103" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="B25" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C25" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>82</v>
+      <c r="B25" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="105" customHeight="1" x14ac:dyDescent="0.2">
@@ -1143,48 +1140,62 @@
         <v>87</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>86</v>
+        <v>78</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="43" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="85" x14ac:dyDescent="0.2">
+      <c r="A28" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="105" x14ac:dyDescent="0.2">
+      <c r="A29" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C29" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D29" s="7" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="43" x14ac:dyDescent="0.2">
-      <c r="A28" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="B28" s="6" t="s">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="B30" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="D28" s="8" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B29" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="C29" s="11"/>
+      <c r="C30" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>